<commit_message>
fix(templates): add required Module column to Ruleset Mapping Entitlement-to-Privilege sheet
Both client_ruleset_template.xlsx and ey_ruleset_template.xlsx were missing
the Module column on 'Entitlement to Privilege', which SHEET_REQUIRED_COLS
in routers/ruleset_mapping.py has required since the module-aware confidence
scoring change. Uploading the old templates as-is failed validation.
Regenerated both files with openpyxl, matching the existing template's
navy-header style, and added the corresponding row to each file's
'How to Fill Data' guide sheet.
</commit_message>
<xml_diff>
--- a/backend/templates/ruleset-mapping/client_ruleset_template.xlsx
+++ b/backend/templates/ruleset-mapping/client_ruleset_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SoD Ruleset" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="SA Ruleset" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Entitlement to Privilege" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How to Fill Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoD Ruleset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA Ruleset" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entitlement to Privilege" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Fill Data" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <sz val="10"/>
     </font>
   </fonts>
@@ -111,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,6 +148,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -613,12 +634,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -635,6 +657,11 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Privilege Code</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Module</t>
         </is>
       </c>
     </row>
@@ -656,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -670,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -705,6 +733,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -791,6 +820,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
@@ -877,6 +907,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
@@ -936,6 +967,18 @@
       <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Oracle privilege code (e.g. ORA_PO_CREATE). Must be consistent across both files for matching to work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Oracle module this privilege belongs to (e.g. Payables). Required — used to improve match accuracy between Client and EY entitlements.</t>
         </is>
       </c>
     </row>

</xml_diff>